<commit_message>
5th Last commit in testing-updated and added missing files.
</commit_message>
<xml_diff>
--- a/IAC IP25 - Machine Learning - Project Schedule - Pranay Sunil Jagtap.xlsx
+++ b/IAC IP25 - Machine Learning - Project Schedule - Pranay Sunil Jagtap.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
@@ -9,7 +9,7 @@
   </bookViews>
   <sheets>
     <sheet name="Guide" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="EXAMPLE" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Machine Learning - Project Sche" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <externalReferences>
     <externalReference r:id="rId5"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="71">
   <si>
     <t xml:space="preserve">IAC INTERNSHIP PROGRAM 2023</t>
   </si>
@@ -184,7 +184,10 @@
     <t xml:space="preserve">          1.3 Create a project charter</t>
   </si>
   <si>
-    <t xml:space="preserve">          1.4 Requirement gathering (SRS)</t>
+    <t xml:space="preserve">          1.4 Requirement Elicitation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">          1.5 Requirement gathering (SRS)</t>
   </si>
   <si>
     <t xml:space="preserve">Planning</t>
@@ -646,6 +649,10 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -780,10 +787,6 @@
     </xf>
     <xf numFmtId="164" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -979,8 +982,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table215" displayName="Table215" ref="A13:G91" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A13:G91"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table215" displayName="Table215" ref="A13:G92" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A13:G92"/>
   <tableColumns count="7">
     <tableColumn id="1" name="SL NO"/>
     <tableColumn id="2" name="TASK NAME"/>
@@ -1179,95 +1182,95 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="21.43"/>
   </cols>
   <sheetData>
-    <row r="2" customFormat="false" ht="17.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="4" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="4" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="3" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="1" t="s">
+      <c r="A7" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="4" t="n">
+      <c r="B7" s="5" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="5" t="s">
+      <c r="A10" s="6" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="6" t="s">
+      <c r="A11" s="7" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="6" t="s">
+      <c r="A12" s="7" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="6" t="s">
+      <c r="A13" s="7" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="7" t="s">
+      <c r="A14" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="B14" s="8"/>
-      <c r="C14" s="8"/>
-      <c r="D14" s="8"/>
-      <c r="E14" s="8"/>
-      <c r="F14" s="8"/>
-      <c r="G14" s="8"/>
-    </row>
-    <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="9" t="s">
+      <c r="B14" s="9"/>
+      <c r="C14" s="9"/>
+      <c r="D14" s="9"/>
+      <c r="E14" s="9"/>
+      <c r="F14" s="9"/>
+      <c r="G14" s="9"/>
+    </row>
+    <row r="16" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="B16" s="8"/>
-      <c r="C16" s="8"/>
-      <c r="D16" s="8"/>
-      <c r="E16" s="8"/>
-      <c r="F16" s="8"/>
-      <c r="G16" s="8"/>
-      <c r="H16" s="8"/>
-      <c r="I16" s="8"/>
-      <c r="J16" s="8"/>
-      <c r="K16" s="8"/>
-      <c r="L16" s="8"/>
-      <c r="M16" s="8"/>
-      <c r="N16" s="8"/>
-      <c r="O16" s="8"/>
+      <c r="B16" s="9"/>
+      <c r="C16" s="9"/>
+      <c r="D16" s="9"/>
+      <c r="E16" s="9"/>
+      <c r="F16" s="9"/>
+      <c r="G16" s="9"/>
+      <c r="H16" s="9"/>
+      <c r="I16" s="9"/>
+      <c r="J16" s="9"/>
+      <c r="K16" s="9"/>
+      <c r="L16" s="9"/>
+      <c r="M16" s="9"/>
+      <c r="N16" s="9"/>
+      <c r="O16" s="9"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E31" s="3"/>
+      <c r="E31" s="4"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -1289,1234 +1292,1260 @@
     <tabColor rgb="FFFFC000"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R98"/>
+  <dimension ref="A1:R99"/>
   <sheetFormatPr defaultColWidth="8.859375" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="2" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="10" width="21.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="11" width="21.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="76.14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="17.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="10" width="18.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="10" width="18.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="11" width="18.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="11" width="18.29"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="18.29"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="17.43"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="24" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="11" t="s">
+    <row r="1" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12"/>
     </row>
     <row r="2" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="12"/>
-      <c r="G2" s="12"/>
-      <c r="I2" s="13" t="s">
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
+      <c r="F2" s="13"/>
+      <c r="G2" s="13"/>
+      <c r="I2" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="J2" s="13"/>
-      <c r="K2" s="13"/>
-      <c r="L2" s="13"/>
-      <c r="M2" s="13"/>
-      <c r="N2" s="13"/>
-      <c r="O2" s="13"/>
-      <c r="P2" s="13"/>
-      <c r="Q2" s="13"/>
-      <c r="R2" s="13"/>
+      <c r="J2" s="14"/>
+      <c r="K2" s="14"/>
+      <c r="L2" s="14"/>
+      <c r="M2" s="14"/>
+      <c r="N2" s="14"/>
+      <c r="O2" s="14"/>
+      <c r="P2" s="14"/>
+      <c r="Q2" s="14"/>
+      <c r="R2" s="14"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I3" s="13"/>
-      <c r="J3" s="13"/>
-      <c r="K3" s="13"/>
-      <c r="L3" s="13"/>
-      <c r="M3" s="13"/>
-      <c r="N3" s="13"/>
-      <c r="O3" s="13"/>
-      <c r="P3" s="13"/>
-      <c r="Q3" s="13"/>
-      <c r="R3" s="13"/>
+      <c r="I3" s="14"/>
+      <c r="J3" s="14"/>
+      <c r="K3" s="14"/>
+      <c r="L3" s="14"/>
+      <c r="M3" s="14"/>
+      <c r="N3" s="14"/>
+      <c r="O3" s="14"/>
+      <c r="P3" s="14"/>
+      <c r="Q3" s="14"/>
+      <c r="R3" s="14"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="14" t="s">
+      <c r="A4" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="15" t="s">
+      <c r="B4" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="E4" s="16" t="s">
+      <c r="E4" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="F4" s="16"/>
-      <c r="G4" s="16"/>
-      <c r="I4" s="13"/>
-      <c r="J4" s="13"/>
-      <c r="K4" s="13"/>
-      <c r="L4" s="13"/>
-      <c r="M4" s="13"/>
-      <c r="N4" s="13"/>
-      <c r="O4" s="13"/>
-      <c r="P4" s="13"/>
-      <c r="Q4" s="13"/>
-      <c r="R4" s="13"/>
+      <c r="F4" s="17"/>
+      <c r="G4" s="17"/>
+      <c r="I4" s="14"/>
+      <c r="J4" s="14"/>
+      <c r="K4" s="14"/>
+      <c r="L4" s="14"/>
+      <c r="M4" s="14"/>
+      <c r="N4" s="14"/>
+      <c r="O4" s="14"/>
+      <c r="P4" s="14"/>
+      <c r="Q4" s="14"/>
+      <c r="R4" s="14"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="17" t="s">
+      <c r="A5" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="B5" s="18" t="s">
+      <c r="B5" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="E5" s="16"/>
-      <c r="F5" s="16"/>
-      <c r="G5" s="16"/>
-      <c r="I5" s="13"/>
-      <c r="J5" s="13"/>
-      <c r="K5" s="13"/>
-      <c r="L5" s="13"/>
-      <c r="M5" s="13"/>
-      <c r="N5" s="13"/>
-      <c r="O5" s="13"/>
-      <c r="P5" s="13"/>
-      <c r="Q5" s="13"/>
-      <c r="R5" s="13"/>
+      <c r="E5" s="17"/>
+      <c r="F5" s="17"/>
+      <c r="G5" s="17"/>
+      <c r="I5" s="14"/>
+      <c r="J5" s="14"/>
+      <c r="K5" s="14"/>
+      <c r="L5" s="14"/>
+      <c r="M5" s="14"/>
+      <c r="N5" s="14"/>
+      <c r="O5" s="14"/>
+      <c r="P5" s="14"/>
+      <c r="Q5" s="14"/>
+      <c r="R5" s="14"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="17" t="s">
+      <c r="A6" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="B6" s="18" t="s">
+      <c r="B6" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="E6" s="16"/>
-      <c r="F6" s="16"/>
-      <c r="G6" s="16"/>
-      <c r="I6" s="13"/>
-      <c r="J6" s="13"/>
-      <c r="K6" s="13"/>
-      <c r="L6" s="13"/>
-      <c r="M6" s="13"/>
-      <c r="N6" s="13"/>
-      <c r="O6" s="13"/>
-      <c r="P6" s="13"/>
-      <c r="Q6" s="13"/>
-      <c r="R6" s="13"/>
+      <c r="E6" s="17"/>
+      <c r="F6" s="17"/>
+      <c r="G6" s="17"/>
+      <c r="I6" s="14"/>
+      <c r="J6" s="14"/>
+      <c r="K6" s="14"/>
+      <c r="L6" s="14"/>
+      <c r="M6" s="14"/>
+      <c r="N6" s="14"/>
+      <c r="O6" s="14"/>
+      <c r="P6" s="14"/>
+      <c r="Q6" s="14"/>
+      <c r="R6" s="14"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="17" t="s">
+      <c r="A7" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="B7" s="18"/>
-      <c r="I7" s="13"/>
-      <c r="J7" s="13"/>
-      <c r="K7" s="13"/>
-      <c r="L7" s="13"/>
-      <c r="M7" s="13"/>
-      <c r="N7" s="13"/>
-      <c r="O7" s="13"/>
-      <c r="P7" s="13"/>
-      <c r="Q7" s="13"/>
-      <c r="R7" s="13"/>
+      <c r="B7" s="19"/>
+      <c r="I7" s="14"/>
+      <c r="J7" s="14"/>
+      <c r="K7" s="14"/>
+      <c r="L7" s="14"/>
+      <c r="M7" s="14"/>
+      <c r="N7" s="14"/>
+      <c r="O7" s="14"/>
+      <c r="P7" s="14"/>
+      <c r="Q7" s="14"/>
+      <c r="R7" s="14"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="17" t="s">
+      <c r="A8" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="B8" s="19" t="n">
+      <c r="B8" s="20" t="n">
         <v>45723</v>
       </c>
-      <c r="I8" s="13"/>
-      <c r="J8" s="13"/>
-      <c r="K8" s="13"/>
-      <c r="L8" s="13"/>
-      <c r="M8" s="13"/>
-      <c r="N8" s="13"/>
-      <c r="O8" s="13"/>
-      <c r="P8" s="13"/>
-      <c r="Q8" s="13"/>
-      <c r="R8" s="13"/>
+      <c r="I8" s="14"/>
+      <c r="J8" s="14"/>
+      <c r="K8" s="14"/>
+      <c r="L8" s="14"/>
+      <c r="M8" s="14"/>
+      <c r="N8" s="14"/>
+      <c r="O8" s="14"/>
+      <c r="P8" s="14"/>
+      <c r="Q8" s="14"/>
+      <c r="R8" s="14"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="17" t="s">
+      <c r="A9" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="B9" s="19" t="n">
+      <c r="B9" s="20" t="n">
         <v>43942</v>
       </c>
-      <c r="I9" s="13"/>
-      <c r="J9" s="13"/>
-      <c r="K9" s="13"/>
-      <c r="L9" s="13"/>
-      <c r="M9" s="13"/>
-      <c r="N9" s="13"/>
-      <c r="O9" s="13"/>
-      <c r="P9" s="13"/>
-      <c r="Q9" s="13"/>
-      <c r="R9" s="13"/>
+      <c r="I9" s="14"/>
+      <c r="J9" s="14"/>
+      <c r="K9" s="14"/>
+      <c r="L9" s="14"/>
+      <c r="M9" s="14"/>
+      <c r="N9" s="14"/>
+      <c r="O9" s="14"/>
+      <c r="P9" s="14"/>
+      <c r="Q9" s="14"/>
+      <c r="R9" s="14"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="20" t="s">
+      <c r="A10" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="B10" s="21" t="s">
+      <c r="B10" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="I10" s="13"/>
-      <c r="J10" s="13"/>
-      <c r="K10" s="13"/>
-      <c r="L10" s="13"/>
-      <c r="M10" s="13"/>
-      <c r="N10" s="13"/>
-      <c r="O10" s="13"/>
-      <c r="P10" s="13"/>
-      <c r="Q10" s="13"/>
-      <c r="R10" s="13"/>
+      <c r="I10" s="14"/>
+      <c r="J10" s="14"/>
+      <c r="K10" s="14"/>
+      <c r="L10" s="14"/>
+      <c r="M10" s="14"/>
+      <c r="N10" s="14"/>
+      <c r="O10" s="14"/>
+      <c r="P10" s="14"/>
+      <c r="Q10" s="14"/>
+      <c r="R10" s="14"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I11" s="13"/>
-      <c r="J11" s="13"/>
-      <c r="K11" s="13"/>
-      <c r="L11" s="13"/>
-      <c r="M11" s="13"/>
-      <c r="N11" s="13"/>
-      <c r="O11" s="13"/>
-      <c r="P11" s="13"/>
-      <c r="Q11" s="13"/>
-      <c r="R11" s="13"/>
+      <c r="I11" s="14"/>
+      <c r="J11" s="14"/>
+      <c r="K11" s="14"/>
+      <c r="L11" s="14"/>
+      <c r="M11" s="14"/>
+      <c r="N11" s="14"/>
+      <c r="O11" s="14"/>
+      <c r="P11" s="14"/>
+      <c r="Q11" s="14"/>
+      <c r="R11" s="14"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I12" s="13"/>
-      <c r="J12" s="13"/>
-      <c r="K12" s="13"/>
-      <c r="L12" s="13"/>
-      <c r="M12" s="13"/>
-      <c r="N12" s="13"/>
-      <c r="O12" s="13"/>
-      <c r="P12" s="13"/>
-      <c r="Q12" s="13"/>
-      <c r="R12" s="13"/>
-    </row>
-    <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="22" t="s">
+      <c r="I12" s="14"/>
+      <c r="J12" s="14"/>
+      <c r="K12" s="14"/>
+      <c r="L12" s="14"/>
+      <c r="M12" s="14"/>
+      <c r="N12" s="14"/>
+      <c r="O12" s="14"/>
+      <c r="P12" s="14"/>
+      <c r="Q12" s="14"/>
+      <c r="R12" s="14"/>
+    </row>
+    <row r="13" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="23" t="s">
         <v>29</v>
       </c>
-      <c r="B13" s="23" t="s">
+      <c r="B13" s="24" t="s">
         <v>30</v>
       </c>
-      <c r="C13" s="23" t="s">
+      <c r="C13" s="24" t="s">
         <v>31</v>
       </c>
-      <c r="D13" s="24" t="s">
+      <c r="D13" s="25" t="s">
         <v>32</v>
       </c>
-      <c r="E13" s="24" t="s">
+      <c r="E13" s="25" t="s">
         <v>33</v>
       </c>
-      <c r="F13" s="23" t="s">
+      <c r="F13" s="24" t="s">
         <v>34</v>
       </c>
-      <c r="G13" s="23" t="s">
+      <c r="G13" s="24" t="s">
         <v>35</v>
       </c>
-      <c r="I13" s="13"/>
-      <c r="J13" s="13"/>
-      <c r="K13" s="13"/>
-      <c r="L13" s="13"/>
-      <c r="M13" s="13"/>
-      <c r="N13" s="13"/>
-      <c r="O13" s="13"/>
-      <c r="P13" s="13"/>
-      <c r="Q13" s="13"/>
-      <c r="R13" s="13"/>
+      <c r="I13" s="14"/>
+      <c r="J13" s="14"/>
+      <c r="K13" s="14"/>
+      <c r="L13" s="14"/>
+      <c r="M13" s="14"/>
+      <c r="N13" s="14"/>
+      <c r="O13" s="14"/>
+      <c r="P13" s="14"/>
+      <c r="Q13" s="14"/>
+      <c r="R13" s="14"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="25"/>
-      <c r="B14" s="26"/>
-      <c r="C14" s="27"/>
-      <c r="D14" s="28"/>
-      <c r="E14" s="28"/>
-      <c r="F14" s="27"/>
-      <c r="I14" s="13"/>
-      <c r="J14" s="13"/>
-      <c r="K14" s="13"/>
-      <c r="L14" s="13"/>
-      <c r="M14" s="13"/>
-      <c r="N14" s="13"/>
-      <c r="O14" s="13"/>
-      <c r="P14" s="13"/>
-      <c r="Q14" s="13"/>
-      <c r="R14" s="13"/>
-    </row>
-    <row r="15" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="29" t="n">
+      <c r="A14" s="26"/>
+      <c r="B14" s="27"/>
+      <c r="C14" s="28"/>
+      <c r="D14" s="29"/>
+      <c r="E14" s="29"/>
+      <c r="F14" s="28"/>
+      <c r="I14" s="14"/>
+      <c r="J14" s="14"/>
+      <c r="K14" s="14"/>
+      <c r="L14" s="14"/>
+      <c r="M14" s="14"/>
+      <c r="N14" s="14"/>
+      <c r="O14" s="14"/>
+      <c r="P14" s="14"/>
+      <c r="Q14" s="14"/>
+      <c r="R14" s="14"/>
+    </row>
+    <row r="15" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="B15" s="30" t="s">
+      <c r="B15" s="31" t="s">
         <v>36</v>
       </c>
-      <c r="C15" s="31" t="s">
-        <v>37</v>
-      </c>
-      <c r="D15" s="32" t="n">
+      <c r="C15" s="32" t="s">
+        <v>37</v>
+      </c>
+      <c r="D15" s="33" t="n">
         <v>45723</v>
       </c>
-      <c r="E15" s="33" t="n">
+      <c r="E15" s="34" t="n">
         <v>45723</v>
       </c>
-      <c r="F15" s="26" t="n">
+      <c r="F15" s="27" t="n">
         <v>1</v>
       </c>
       <c r="G15" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="I15" s="13"/>
-      <c r="J15" s="13"/>
-      <c r="K15" s="13"/>
-      <c r="L15" s="13"/>
-      <c r="M15" s="13"/>
-      <c r="N15" s="13"/>
-      <c r="O15" s="13"/>
-      <c r="P15" s="13"/>
-      <c r="Q15" s="13"/>
-      <c r="R15" s="13"/>
-    </row>
-    <row r="16" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="25"/>
-      <c r="B16" s="34" t="s">
+      <c r="I15" s="14"/>
+      <c r="J15" s="14"/>
+      <c r="K15" s="14"/>
+      <c r="L15" s="14"/>
+      <c r="M15" s="14"/>
+      <c r="N15" s="14"/>
+      <c r="O15" s="14"/>
+      <c r="P15" s="14"/>
+      <c r="Q15" s="14"/>
+      <c r="R15" s="14"/>
+    </row>
+    <row r="16" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="26"/>
+      <c r="B16" s="35" t="s">
         <v>39</v>
       </c>
-      <c r="C16" s="31" t="s">
-        <v>37</v>
-      </c>
-      <c r="D16" s="35" t="n">
+      <c r="C16" s="32" t="s">
+        <v>37</v>
+      </c>
+      <c r="D16" s="36" t="n">
         <v>45723</v>
       </c>
-      <c r="E16" s="35" t="n">
+      <c r="E16" s="36" t="n">
         <v>45723</v>
       </c>
-      <c r="F16" s="27" t="n">
+      <c r="F16" s="28" t="n">
         <v>1</v>
       </c>
       <c r="G16" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="I16" s="13"/>
-      <c r="J16" s="13"/>
-      <c r="K16" s="13"/>
-      <c r="L16" s="13"/>
-      <c r="M16" s="13"/>
-      <c r="N16" s="13"/>
-      <c r="O16" s="13"/>
-      <c r="P16" s="13"/>
-      <c r="Q16" s="13"/>
-      <c r="R16" s="13"/>
-    </row>
-    <row r="17" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A17" s="36"/>
-      <c r="B17" s="1" t="s">
+      <c r="I16" s="14"/>
+      <c r="J16" s="14"/>
+      <c r="K16" s="14"/>
+      <c r="L16" s="14"/>
+      <c r="M16" s="14"/>
+      <c r="N16" s="14"/>
+      <c r="O16" s="14"/>
+      <c r="P16" s="14"/>
+      <c r="Q16" s="14"/>
+      <c r="R16" s="14"/>
+    </row>
+    <row r="17" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A17" s="37"/>
+      <c r="B17" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="C17" s="31" t="s">
-        <v>37</v>
-      </c>
-      <c r="D17" s="35" t="n">
+      <c r="C17" s="32" t="s">
+        <v>37</v>
+      </c>
+      <c r="D17" s="36" t="n">
         <v>45723</v>
       </c>
-      <c r="E17" s="35" t="n">
+      <c r="E17" s="36" t="n">
         <v>45723</v>
       </c>
-      <c r="F17" s="27" t="n">
+      <c r="F17" s="28" t="n">
         <v>1</v>
       </c>
       <c r="G17" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="I17" s="13"/>
-      <c r="J17" s="13"/>
-      <c r="K17" s="13"/>
-      <c r="L17" s="13"/>
-      <c r="M17" s="13"/>
-      <c r="N17" s="13"/>
-      <c r="O17" s="13"/>
-      <c r="P17" s="13"/>
-      <c r="Q17" s="13"/>
-      <c r="R17" s="13"/>
-    </row>
-    <row r="18" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A18" s="25"/>
-      <c r="B18" s="1" t="s">
+      <c r="I17" s="14"/>
+      <c r="J17" s="14"/>
+      <c r="K17" s="14"/>
+      <c r="L17" s="14"/>
+      <c r="M17" s="14"/>
+      <c r="N17" s="14"/>
+      <c r="O17" s="14"/>
+      <c r="P17" s="14"/>
+      <c r="Q17" s="14"/>
+      <c r="R17" s="14"/>
+    </row>
+    <row r="18" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A18" s="26"/>
+      <c r="B18" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="C18" s="31" t="s">
-        <v>37</v>
-      </c>
-      <c r="D18" s="35" t="n">
+      <c r="C18" s="32" t="s">
+        <v>37</v>
+      </c>
+      <c r="D18" s="36" t="n">
         <v>45723</v>
       </c>
-      <c r="E18" s="35" t="n">
+      <c r="E18" s="36" t="n">
         <v>45723</v>
       </c>
-      <c r="F18" s="27" t="n">
+      <c r="F18" s="28" t="n">
         <v>1</v>
       </c>
       <c r="G18" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="I18" s="13"/>
-      <c r="J18" s="13"/>
-      <c r="K18" s="13"/>
-      <c r="L18" s="13"/>
-      <c r="M18" s="13"/>
-      <c r="N18" s="13"/>
-      <c r="O18" s="13"/>
-      <c r="P18" s="13"/>
-      <c r="Q18" s="13"/>
-      <c r="R18" s="13"/>
-    </row>
-    <row r="19" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A19" s="36"/>
-      <c r="B19" s="1" t="s">
+      <c r="I18" s="14"/>
+      <c r="J18" s="14"/>
+      <c r="K18" s="14"/>
+      <c r="L18" s="14"/>
+      <c r="M18" s="14"/>
+      <c r="N18" s="14"/>
+      <c r="O18" s="14"/>
+      <c r="P18" s="14"/>
+      <c r="Q18" s="14"/>
+      <c r="R18" s="14"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A19" s="26"/>
+      <c r="B19" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="C19" s="31" t="s">
-        <v>37</v>
-      </c>
-      <c r="D19" s="35" t="n">
+      <c r="C19" s="32" t="s">
+        <v>37</v>
+      </c>
+      <c r="D19" s="36" t="n">
         <v>45723</v>
       </c>
-      <c r="E19" s="35" t="n">
+      <c r="E19" s="36" t="n">
         <v>45723</v>
       </c>
-      <c r="F19" s="27" t="n">
+      <c r="F19" s="28"/>
+      <c r="I19" s="14"/>
+      <c r="J19" s="14"/>
+      <c r="K19" s="14"/>
+      <c r="L19" s="14"/>
+      <c r="M19" s="14"/>
+      <c r="N19" s="14"/>
+      <c r="O19" s="14"/>
+      <c r="P19" s="14"/>
+      <c r="Q19" s="14"/>
+      <c r="R19" s="14"/>
+    </row>
+    <row r="20" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A20" s="37"/>
+      <c r="B20" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C20" s="32" t="s">
+        <v>37</v>
+      </c>
+      <c r="D20" s="36" t="n">
+        <v>45723</v>
+      </c>
+      <c r="E20" s="36" t="n">
+        <v>45723</v>
+      </c>
+      <c r="F20" s="28" t="n">
         <v>1</v>
       </c>
-      <c r="G19" s="1" t="s">
+      <c r="G20" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="I19" s="13"/>
-      <c r="J19" s="13"/>
-      <c r="K19" s="13"/>
-      <c r="L19" s="13"/>
-      <c r="M19" s="13"/>
-      <c r="N19" s="13"/>
-      <c r="O19" s="13"/>
-      <c r="P19" s="13"/>
-      <c r="Q19" s="13"/>
-      <c r="R19" s="13"/>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="36"/>
-      <c r="I20" s="13"/>
-      <c r="J20" s="13"/>
-      <c r="K20" s="13"/>
-      <c r="L20" s="13"/>
-      <c r="M20" s="13"/>
-      <c r="N20" s="13"/>
-      <c r="O20" s="13"/>
-      <c r="P20" s="13"/>
-      <c r="Q20" s="13"/>
-      <c r="R20" s="13"/>
+      <c r="I20" s="14"/>
+      <c r="J20" s="14"/>
+      <c r="K20" s="14"/>
+      <c r="L20" s="14"/>
+      <c r="M20" s="14"/>
+      <c r="N20" s="14"/>
+      <c r="O20" s="14"/>
+      <c r="P20" s="14"/>
+      <c r="Q20" s="14"/>
+      <c r="R20" s="14"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="36"/>
-      <c r="B21" s="26"/>
-      <c r="I21" s="13"/>
-      <c r="J21" s="13"/>
-      <c r="K21" s="13"/>
-      <c r="L21" s="13"/>
-      <c r="M21" s="13"/>
-      <c r="N21" s="13"/>
-      <c r="O21" s="13"/>
-      <c r="P21" s="13"/>
-      <c r="Q21" s="13"/>
-      <c r="R21" s="13"/>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A22" s="29" t="n">
+      <c r="A21" s="37"/>
+      <c r="I21" s="14"/>
+      <c r="J21" s="14"/>
+      <c r="K21" s="14"/>
+      <c r="L21" s="14"/>
+      <c r="M21" s="14"/>
+      <c r="N21" s="14"/>
+      <c r="O21" s="14"/>
+      <c r="P21" s="14"/>
+      <c r="Q21" s="14"/>
+      <c r="R21" s="14"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="37"/>
+      <c r="B22" s="27"/>
+      <c r="I22" s="14"/>
+      <c r="J22" s="14"/>
+      <c r="K22" s="14"/>
+      <c r="L22" s="14"/>
+      <c r="M22" s="14"/>
+      <c r="N22" s="14"/>
+      <c r="O22" s="14"/>
+      <c r="P22" s="14"/>
+      <c r="Q22" s="14"/>
+      <c r="R22" s="14"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A23" s="30" t="n">
         <v>2</v>
       </c>
-      <c r="B22" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="C22" s="31" t="s">
-        <v>37</v>
-      </c>
-      <c r="D22" s="32" t="n">
+      <c r="B23" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="C23" s="32" t="s">
+        <v>37</v>
+      </c>
+      <c r="D23" s="33" t="n">
         <v>45726</v>
       </c>
-      <c r="E22" s="32" t="n">
-        <v>45726</v>
-      </c>
-      <c r="F22" s="26" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A23" s="36"/>
-      <c r="B23" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="C23" s="31" t="s">
-        <v>37</v>
-      </c>
-      <c r="D23" s="35" t="n">
-        <v>45726</v>
-      </c>
-      <c r="E23" s="35" t="n">
+      <c r="E23" s="33" t="n">
         <v>45726</v>
       </c>
       <c r="F23" s="27" t="n">
         <v>1</v>
       </c>
-      <c r="G23" s="1" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A24" s="36"/>
-      <c r="B24" s="1" t="s">
+    </row>
+    <row r="24" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A24" s="37"/>
+      <c r="B24" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="C24" s="31" t="s">
-        <v>37</v>
-      </c>
-      <c r="D24" s="35" t="n">
+      <c r="C24" s="32" t="s">
+        <v>37</v>
+      </c>
+      <c r="D24" s="36" t="n">
         <v>45726</v>
       </c>
-      <c r="E24" s="35" t="n">
+      <c r="E24" s="36" t="n">
         <v>45726</v>
       </c>
-      <c r="F24" s="27" t="n">
+      <c r="F24" s="28" t="n">
         <v>1</v>
       </c>
       <c r="G24" s="1" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A25" s="36"/>
-      <c r="B25" s="1" t="s">
+    <row r="25" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A25" s="37"/>
+      <c r="B25" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="C25" s="31" t="s">
-        <v>37</v>
-      </c>
-      <c r="D25" s="35" t="n">
+      <c r="C25" s="32" t="s">
+        <v>37</v>
+      </c>
+      <c r="D25" s="36" t="n">
         <v>45726</v>
       </c>
-      <c r="E25" s="35" t="n">
+      <c r="E25" s="36" t="n">
         <v>45726</v>
       </c>
-      <c r="F25" s="27" t="n">
+      <c r="F25" s="28" t="n">
         <v>1</v>
       </c>
       <c r="G25" s="1" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A26" s="36"/>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="36"/>
-    </row>
-    <row r="28" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="29" t="n">
+    <row r="26" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A26" s="37"/>
+      <c r="B26" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C26" s="32" t="s">
+        <v>37</v>
+      </c>
+      <c r="D26" s="36" t="n">
+        <v>45726</v>
+      </c>
+      <c r="E26" s="36" t="n">
+        <v>45726</v>
+      </c>
+      <c r="F26" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="G26" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A27" s="37"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="37"/>
+    </row>
+    <row r="29" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="30" t="n">
         <v>3</v>
       </c>
-      <c r="B28" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="C28" s="31" t="s">
-        <v>37</v>
-      </c>
-      <c r="D28" s="32" t="n">
+      <c r="B29" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="C29" s="32" t="s">
+        <v>37</v>
+      </c>
+      <c r="D29" s="33" t="n">
         <v>45727</v>
       </c>
-      <c r="E28" s="32" t="n">
+      <c r="E29" s="33" t="n">
         <v>45765</v>
-      </c>
-      <c r="G28" s="1" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A29" s="36"/>
-      <c r="B29" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="C29" s="31" t="s">
-        <v>37</v>
-      </c>
-      <c r="D29" s="32" t="n">
-        <v>45727</v>
-      </c>
-      <c r="E29" s="32" t="n">
-        <v>45730</v>
-      </c>
-      <c r="F29" s="26" t="n">
-        <v>4</v>
       </c>
       <c r="G29" s="1" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A30" s="36"/>
-      <c r="B30" s="3" t="s">
+    <row r="30" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A30" s="37"/>
+      <c r="B30" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="C30" s="31" t="s">
-        <v>37</v>
-      </c>
-      <c r="D30" s="35" t="n">
+      <c r="C30" s="32" t="s">
+        <v>37</v>
+      </c>
+      <c r="D30" s="33" t="n">
         <v>45727</v>
       </c>
-      <c r="E30" s="35" t="n">
+      <c r="E30" s="33" t="n">
+        <v>45730</v>
+      </c>
+      <c r="F30" s="27" t="n">
+        <v>4</v>
+      </c>
+      <c r="G30" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A31" s="37"/>
+      <c r="B31" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C31" s="32" t="s">
+        <v>37</v>
+      </c>
+      <c r="D31" s="36" t="n">
         <v>45727</v>
       </c>
-      <c r="F30" s="27" t="n">
+      <c r="E31" s="36" t="n">
+        <v>45727</v>
+      </c>
+      <c r="F31" s="28" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A31" s="36"/>
-      <c r="B31" s="37" t="s">
-        <v>50</v>
-      </c>
-      <c r="C31" s="31" t="s">
-        <v>37</v>
-      </c>
-      <c r="D31" s="35"/>
-      <c r="E31" s="35"/>
-      <c r="F31" s="27"/>
-    </row>
-    <row r="32" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A32" s="36"/>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A32" s="37"/>
       <c r="B32" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="C32" s="31" t="s">
-        <v>37</v>
-      </c>
-      <c r="D32" s="35" t="n">
+      <c r="C32" s="32" t="s">
+        <v>37</v>
+      </c>
+      <c r="D32" s="36"/>
+      <c r="E32" s="36"/>
+      <c r="F32" s="28"/>
+    </row>
+    <row r="33" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A33" s="37"/>
+      <c r="B33" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C33" s="32" t="s">
+        <v>37</v>
+      </c>
+      <c r="D33" s="36" t="n">
         <v>45728</v>
       </c>
-      <c r="E32" s="35" t="n">
+      <c r="E33" s="36" t="n">
         <v>45729</v>
       </c>
-      <c r="F32" s="27" t="n">
+      <c r="F33" s="28" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A33" s="36"/>
-      <c r="B33" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="C33" s="31" t="s">
-        <v>37</v>
-      </c>
-      <c r="D33" s="35" t="n">
+    <row r="34" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A34" s="37"/>
+      <c r="B34" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="C34" s="32" t="s">
+        <v>37</v>
+      </c>
+      <c r="D34" s="36" t="n">
         <v>45730</v>
       </c>
-      <c r="E33" s="35" t="n">
+      <c r="E34" s="36" t="n">
         <v>45730</v>
       </c>
-      <c r="F33" s="27" t="n">
+      <c r="F34" s="28" t="n">
         <v>1</v>
       </c>
-      <c r="G33" s="1" t="s">
+      <c r="G34" s="1" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A34" s="36"/>
-      <c r="B34" s="37" t="s">
-        <v>53</v>
-      </c>
-      <c r="C34" s="31" t="s">
-        <v>37</v>
-      </c>
-      <c r="D34" s="35"/>
-      <c r="E34" s="35"/>
-      <c r="F34" s="27"/>
-    </row>
-    <row r="35" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
-      <c r="A35" s="36"/>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A35" s="37"/>
       <c r="B35" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="C35" s="31" t="s">
-        <v>37</v>
-      </c>
-      <c r="D35" s="32" t="n">
+      <c r="C35" s="32" t="s">
+        <v>37</v>
+      </c>
+      <c r="D35" s="36"/>
+      <c r="E35" s="36"/>
+      <c r="F35" s="28"/>
+    </row>
+    <row r="36" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
+      <c r="A36" s="37"/>
+      <c r="B36" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="C36" s="32" t="s">
+        <v>37</v>
+      </c>
+      <c r="D36" s="33" t="n">
         <v>45733</v>
       </c>
-      <c r="E35" s="32" t="n">
+      <c r="E36" s="33" t="n">
         <v>45754</v>
       </c>
-      <c r="F35" s="26" t="n">
+      <c r="F36" s="27" t="n">
         <v>16</v>
-      </c>
-      <c r="G35" s="1" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
-      <c r="A36" s="36"/>
-      <c r="B36" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="C36" s="31" t="s">
-        <v>37</v>
-      </c>
-      <c r="D36" s="32" t="n">
-        <v>45733</v>
-      </c>
-      <c r="E36" s="32" t="n">
-        <v>45747</v>
-      </c>
-      <c r="F36" s="27" t="n">
-        <v>11</v>
       </c>
       <c r="G36" s="1" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
-      <c r="A37" s="36"/>
-      <c r="B37" s="3" t="s">
+    <row r="37" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
+      <c r="A37" s="37"/>
+      <c r="B37" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="C37" s="31" t="s">
-        <v>37</v>
-      </c>
-      <c r="D37" s="32" t="n">
+      <c r="C37" s="32" t="s">
+        <v>37</v>
+      </c>
+      <c r="D37" s="33" t="n">
         <v>45733</v>
       </c>
-      <c r="E37" s="32" t="n">
-        <v>45737</v>
-      </c>
-      <c r="F37" s="27" t="n">
-        <v>5</v>
+      <c r="E37" s="33" t="n">
+        <v>45747</v>
+      </c>
+      <c r="F37" s="28" t="n">
+        <v>11</v>
       </c>
       <c r="G37" s="1" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
-      <c r="A38" s="36"/>
-      <c r="B38" s="1" t="s">
+    <row r="38" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
+      <c r="A38" s="37"/>
+      <c r="B38" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="C38" s="31" t="s">
-        <v>37</v>
-      </c>
-      <c r="D38" s="32"/>
-      <c r="E38" s="32"/>
+      <c r="C38" s="32" t="s">
+        <v>37</v>
+      </c>
+      <c r="D38" s="33" t="n">
+        <v>45733</v>
+      </c>
+      <c r="E38" s="33" t="n">
+        <v>45737</v>
+      </c>
+      <c r="F38" s="28" t="n">
+        <v>5</v>
+      </c>
+      <c r="G38" s="1" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
-      <c r="A39" s="36"/>
-      <c r="B39" s="1" t="s">
+      <c r="A39" s="37"/>
+      <c r="B39" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="C39" s="31" t="s">
-        <v>37</v>
-      </c>
-      <c r="D39" s="32"/>
-      <c r="E39" s="32"/>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A40" s="36"/>
-      <c r="B40" s="37" t="s">
+      <c r="C39" s="32" t="s">
+        <v>37</v>
+      </c>
+      <c r="D39" s="33"/>
+      <c r="E39" s="33"/>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
+      <c r="A40" s="37"/>
+      <c r="B40" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="C40" s="31" t="s">
-        <v>37</v>
-      </c>
-      <c r="D40" s="32"/>
-      <c r="E40" s="32"/>
-      <c r="F40" s="27"/>
+      <c r="C40" s="32" t="s">
+        <v>37</v>
+      </c>
+      <c r="D40" s="33"/>
+      <c r="E40" s="33"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A41" s="36"/>
-      <c r="B41" s="37" t="s">
+      <c r="A41" s="37"/>
+      <c r="B41" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="C41" s="31" t="s">
-        <v>37</v>
-      </c>
-      <c r="D41" s="32"/>
-      <c r="E41" s="32"/>
-      <c r="F41" s="27"/>
-    </row>
-    <row r="42" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A42" s="36"/>
+      <c r="C41" s="32" t="s">
+        <v>37</v>
+      </c>
+      <c r="D41" s="33"/>
+      <c r="E41" s="33"/>
+      <c r="F41" s="28"/>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A42" s="37"/>
       <c r="B42" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="C42" s="31" t="s">
-        <v>37</v>
-      </c>
-      <c r="D42" s="32" t="n">
+      <c r="C42" s="32" t="s">
+        <v>37</v>
+      </c>
+      <c r="D42" s="33"/>
+      <c r="E42" s="33"/>
+      <c r="F42" s="28"/>
+    </row>
+    <row r="43" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A43" s="37"/>
+      <c r="B43" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="C43" s="32" t="s">
+        <v>37</v>
+      </c>
+      <c r="D43" s="33" t="n">
         <v>45740</v>
       </c>
-      <c r="E42" s="32" t="n">
+      <c r="E43" s="33" t="n">
         <v>45744</v>
       </c>
-      <c r="F42" s="27" t="n">
+      <c r="F43" s="28" t="n">
         <v>5</v>
       </c>
-      <c r="G42" s="1" t="s">
+      <c r="G43" s="1" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A43" s="36"/>
-      <c r="B43" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="C43" s="31" t="s">
-        <v>37</v>
-      </c>
-      <c r="D43" s="32"/>
-      <c r="E43" s="32"/>
-      <c r="F43" s="27"/>
-    </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A44" s="36"/>
-      <c r="B44" s="1" t="s">
+      <c r="A44" s="37"/>
+      <c r="B44" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="C44" s="31" t="s">
-        <v>37</v>
-      </c>
-      <c r="D44" s="32"/>
-      <c r="E44" s="32"/>
-      <c r="F44" s="27"/>
+      <c r="C44" s="32" t="s">
+        <v>37</v>
+      </c>
+      <c r="D44" s="33"/>
+      <c r="E44" s="33"/>
+      <c r="F44" s="28"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A45" s="36"/>
-      <c r="B45" s="37" t="s">
+      <c r="A45" s="37"/>
+      <c r="B45" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="C45" s="31" t="s">
-        <v>37</v>
-      </c>
-      <c r="D45" s="32"/>
-      <c r="E45" s="32"/>
-      <c r="F45" s="27"/>
+      <c r="C45" s="32" t="s">
+        <v>37</v>
+      </c>
+      <c r="D45" s="33"/>
+      <c r="E45" s="33"/>
+      <c r="F45" s="28"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A46" s="36"/>
-      <c r="B46" s="37" t="s">
+      <c r="A46" s="37"/>
+      <c r="B46" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="C46" s="31" t="s">
-        <v>37</v>
-      </c>
-      <c r="D46" s="32"/>
-      <c r="E46" s="32"/>
-    </row>
-    <row r="47" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A47" s="36"/>
-      <c r="B47" s="37" t="s">
-        <v>62</v>
-      </c>
-      <c r="C47" s="31" t="s">
-        <v>37</v>
-      </c>
-      <c r="D47" s="32" t="n">
+      <c r="C46" s="32" t="s">
+        <v>37</v>
+      </c>
+      <c r="D46" s="33"/>
+      <c r="E46" s="33"/>
+      <c r="F46" s="28"/>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A47" s="37"/>
+      <c r="B47" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C47" s="32" t="s">
+        <v>37</v>
+      </c>
+      <c r="D47" s="33"/>
+      <c r="E47" s="33"/>
+    </row>
+    <row r="48" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A48" s="37"/>
+      <c r="B48" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="C48" s="32" t="s">
+        <v>37</v>
+      </c>
+      <c r="D48" s="33" t="n">
         <v>45747</v>
       </c>
-      <c r="E47" s="32" t="n">
+      <c r="E48" s="33" t="n">
         <v>45747</v>
       </c>
-      <c r="F47" s="27" t="n">
+      <c r="F48" s="28" t="n">
         <v>1</v>
-      </c>
-      <c r="G47" s="1" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="48" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
-      <c r="A48" s="36"/>
-      <c r="B48" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="C48" s="31" t="s">
-        <v>37</v>
-      </c>
-      <c r="D48" s="32" t="n">
-        <v>45748</v>
-      </c>
-      <c r="E48" s="32" t="n">
-        <v>45754</v>
-      </c>
-      <c r="F48" s="27" t="n">
-        <v>5</v>
       </c>
       <c r="G48" s="1" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
-      <c r="A49" s="36"/>
-      <c r="B49" s="1" t="s">
+    <row r="49" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
+      <c r="A49" s="37"/>
+      <c r="B49" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="C49" s="31" t="s">
-        <v>37</v>
-      </c>
-      <c r="D49" s="32"/>
-      <c r="E49" s="32"/>
-      <c r="F49" s="27"/>
-    </row>
-    <row r="50" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
-      <c r="A50" s="36"/>
+      <c r="C49" s="32" t="s">
+        <v>37</v>
+      </c>
+      <c r="D49" s="33" t="n">
+        <v>45748</v>
+      </c>
+      <c r="E49" s="33" t="n">
+        <v>45754</v>
+      </c>
+      <c r="F49" s="28" t="n">
+        <v>5</v>
+      </c>
+      <c r="G49" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
+      <c r="A50" s="37"/>
       <c r="B50" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="C50" s="31" t="s">
-        <v>37</v>
-      </c>
-      <c r="D50" s="32" t="n">
+      <c r="C50" s="32" t="s">
+        <v>37</v>
+      </c>
+      <c r="D50" s="33"/>
+      <c r="E50" s="33"/>
+      <c r="F50" s="28"/>
+    </row>
+    <row r="51" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
+      <c r="A51" s="37"/>
+      <c r="B51" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="C51" s="32" t="s">
+        <v>37</v>
+      </c>
+      <c r="D51" s="33" t="n">
         <v>45755</v>
       </c>
-      <c r="E50" s="32" t="n">
+      <c r="E51" s="33" t="n">
         <v>45761</v>
       </c>
-      <c r="F50" s="26" t="n">
+      <c r="F51" s="27" t="n">
         <v>5</v>
       </c>
-      <c r="G50" s="1" t="s">
+      <c r="G51" s="1" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
-      <c r="A51" s="36"/>
-      <c r="B51" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="C51" s="31" t="s">
-        <v>37</v>
-      </c>
-      <c r="D51" s="32"/>
-      <c r="E51" s="32"/>
-      <c r="F51" s="27"/>
-    </row>
-    <row r="52" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
-      <c r="A52" s="36"/>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
+      <c r="A52" s="37"/>
       <c r="B52" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="C52" s="31" t="s">
-        <v>37</v>
-      </c>
-      <c r="D52" s="32" t="n">
+      <c r="C52" s="32" t="s">
+        <v>37</v>
+      </c>
+      <c r="D52" s="33"/>
+      <c r="E52" s="33"/>
+      <c r="F52" s="28"/>
+    </row>
+    <row r="53" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
+      <c r="A53" s="37"/>
+      <c r="B53" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="C53" s="32" t="s">
+        <v>37</v>
+      </c>
+      <c r="D53" s="33" t="n">
         <v>45762</v>
       </c>
-      <c r="E52" s="32" t="n">
+      <c r="E53" s="33" t="n">
         <v>45765</v>
       </c>
-      <c r="F52" s="26" t="n">
+      <c r="F53" s="27" t="n">
         <v>4</v>
       </c>
-      <c r="G52" s="1" t="s">
+      <c r="G53" s="1" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
-      <c r="A53" s="36"/>
-      <c r="B53" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="C53" s="31" t="s">
-        <v>37</v>
-      </c>
-      <c r="D53" s="32"/>
-      <c r="E53" s="32"/>
-      <c r="F53" s="27"/>
-    </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A54" s="36"/>
-      <c r="B54" s="3"/>
-      <c r="D54" s="32"/>
-      <c r="E54" s="32"/>
-      <c r="F54" s="27"/>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
+      <c r="A54" s="37"/>
+      <c r="B54" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C54" s="32" t="s">
+        <v>37</v>
+      </c>
+      <c r="D54" s="33"/>
+      <c r="E54" s="33"/>
+      <c r="F54" s="28"/>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A55" s="36"/>
-      <c r="D55" s="32"/>
-      <c r="E55" s="32"/>
-      <c r="F55" s="27"/>
-    </row>
-    <row r="56" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
-      <c r="A56" s="29" t="n">
+      <c r="A55" s="37"/>
+      <c r="B55" s="4"/>
+      <c r="D55" s="33"/>
+      <c r="E55" s="33"/>
+      <c r="F55" s="28"/>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A56" s="37"/>
+      <c r="D56" s="33"/>
+      <c r="E56" s="33"/>
+      <c r="F56" s="28"/>
+    </row>
+    <row r="57" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
+      <c r="A57" s="30" t="n">
         <v>4</v>
       </c>
-      <c r="B56" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="C56" s="31" t="s">
-        <v>37</v>
-      </c>
-      <c r="D56" s="32" t="n">
+      <c r="B57" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="C57" s="32" t="s">
+        <v>37</v>
+      </c>
+      <c r="D57" s="33" t="n">
         <v>45768</v>
       </c>
-      <c r="E56" s="32" t="n">
+      <c r="E57" s="33" t="n">
         <v>45768</v>
       </c>
-      <c r="F56" s="26" t="n">
+      <c r="F57" s="27" t="n">
         <v>1</v>
       </c>
-      <c r="G56" s="1" t="s">
+      <c r="G57" s="1" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
-      <c r="A57" s="36"/>
-      <c r="D57" s="32"/>
-      <c r="E57" s="32"/>
-      <c r="F57" s="27"/>
-    </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
-      <c r="A58" s="36"/>
-      <c r="B58" s="3"/>
-      <c r="D58" s="32"/>
-      <c r="E58" s="32"/>
-      <c r="F58" s="27"/>
+      <c r="A58" s="37"/>
+      <c r="D58" s="33"/>
+      <c r="E58" s="33"/>
+      <c r="F58" s="28"/>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
-      <c r="A59" s="36"/>
-      <c r="D59" s="32"/>
-      <c r="E59" s="32"/>
-      <c r="F59" s="27"/>
-    </row>
-    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="36"/>
-      <c r="D60" s="32"/>
-      <c r="E60" s="32"/>
-      <c r="F60" s="27"/>
+      <c r="A59" s="37"/>
+      <c r="B59" s="4"/>
+      <c r="D59" s="33"/>
+      <c r="E59" s="33"/>
+      <c r="F59" s="28"/>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="2" collapsed="false">
+      <c r="A60" s="37"/>
+      <c r="D60" s="33"/>
+      <c r="E60" s="33"/>
+      <c r="F60" s="28"/>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="36"/>
-      <c r="D61" s="32"/>
-      <c r="E61" s="32"/>
-      <c r="F61" s="27"/>
-    </row>
-    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A62" s="36"/>
-      <c r="D62" s="32"/>
-      <c r="E62" s="32"/>
-      <c r="F62" s="27"/>
+      <c r="A61" s="37"/>
+      <c r="D61" s="33"/>
+      <c r="E61" s="33"/>
+      <c r="F61" s="28"/>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="37"/>
+      <c r="D62" s="33"/>
+      <c r="E62" s="33"/>
+      <c r="F62" s="28"/>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A63" s="36"/>
-      <c r="D63" s="32"/>
-      <c r="E63" s="32"/>
+      <c r="A63" s="37"/>
+      <c r="D63" s="33"/>
+      <c r="E63" s="33"/>
+      <c r="F63" s="28"/>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A64" s="36"/>
-      <c r="B64" s="3"/>
-      <c r="D64" s="32"/>
-      <c r="E64" s="32"/>
-      <c r="F64" s="27"/>
+      <c r="A64" s="37"/>
+      <c r="D64" s="33"/>
+      <c r="E64" s="33"/>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A65" s="36"/>
-      <c r="D65" s="32"/>
-      <c r="E65" s="32"/>
+      <c r="A65" s="37"/>
+      <c r="B65" s="4"/>
+      <c r="D65" s="33"/>
+      <c r="E65" s="33"/>
+      <c r="F65" s="28"/>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A66" s="36"/>
-      <c r="D66" s="32"/>
-      <c r="E66" s="32"/>
+      <c r="A66" s="37"/>
+      <c r="D66" s="33"/>
+      <c r="E66" s="33"/>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A67" s="36"/>
-      <c r="D67" s="32"/>
-      <c r="E67" s="32"/>
-    </row>
-    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="36"/>
-      <c r="D68" s="32"/>
-      <c r="E68" s="32"/>
+      <c r="A67" s="37"/>
+      <c r="D67" s="33"/>
+      <c r="E67" s="33"/>
+    </row>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A68" s="37"/>
+      <c r="D68" s="33"/>
+      <c r="E68" s="33"/>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="36"/>
-      <c r="D69" s="32"/>
-      <c r="E69" s="32"/>
-    </row>
-    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A70" s="36"/>
-      <c r="D70" s="32"/>
-      <c r="E70" s="32"/>
+      <c r="A69" s="37"/>
+      <c r="D69" s="33"/>
+      <c r="E69" s="33"/>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="37"/>
+      <c r="D70" s="33"/>
+      <c r="E70" s="33"/>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A71" s="36"/>
-      <c r="B71" s="3"/>
-      <c r="D71" s="32"/>
-      <c r="E71" s="32"/>
-      <c r="F71" s="27"/>
+      <c r="A71" s="37"/>
+      <c r="D71" s="33"/>
+      <c r="E71" s="33"/>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A72" s="36"/>
-      <c r="D72" s="32"/>
-      <c r="E72" s="32"/>
-    </row>
-    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="36"/>
-      <c r="D73" s="32"/>
-      <c r="E73" s="32"/>
+      <c r="A72" s="37"/>
+      <c r="B72" s="4"/>
+      <c r="D72" s="33"/>
+      <c r="E72" s="33"/>
+      <c r="F72" s="28"/>
+    </row>
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A73" s="37"/>
+      <c r="D73" s="33"/>
+      <c r="E73" s="33"/>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A74" s="36"/>
-      <c r="D74" s="32"/>
-      <c r="E74" s="32"/>
-    </row>
-    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A75" s="36"/>
-      <c r="B75" s="3"/>
-      <c r="D75" s="32"/>
-      <c r="E75" s="32"/>
-      <c r="F75" s="27"/>
+      <c r="A74" s="37"/>
+      <c r="D74" s="33"/>
+      <c r="E74" s="33"/>
+    </row>
+    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="37"/>
+      <c r="D75" s="33"/>
+      <c r="E75" s="33"/>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A76" s="36"/>
-      <c r="B76" s="3"/>
-      <c r="D76" s="32"/>
-      <c r="E76" s="32"/>
+      <c r="A76" s="37"/>
+      <c r="B76" s="4"/>
+      <c r="D76" s="33"/>
+      <c r="E76" s="33"/>
+      <c r="F76" s="28"/>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
-      <c r="A77" s="36"/>
-      <c r="D77" s="32"/>
-      <c r="E77" s="32"/>
-    </row>
-    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A78" s="36"/>
-      <c r="D78" s="32"/>
-      <c r="E78" s="32"/>
+      <c r="A77" s="37"/>
+      <c r="B77" s="4"/>
+      <c r="D77" s="33"/>
+      <c r="E77" s="33"/>
+    </row>
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="1" collapsed="false">
+      <c r="A78" s="37"/>
+      <c r="D78" s="33"/>
+      <c r="E78" s="33"/>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A79" s="36"/>
-      <c r="D79" s="32"/>
-      <c r="E79" s="32"/>
+      <c r="A79" s="37"/>
+      <c r="D79" s="33"/>
+      <c r="E79" s="33"/>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A80" s="36"/>
-      <c r="D80" s="32"/>
-      <c r="E80" s="32"/>
+      <c r="A80" s="37"/>
+      <c r="D80" s="33"/>
+      <c r="E80" s="33"/>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A81" s="36"/>
-      <c r="B81" s="3"/>
-      <c r="D81" s="32"/>
-      <c r="E81" s="32"/>
-      <c r="F81" s="27"/>
+      <c r="A81" s="37"/>
+      <c r="D81" s="33"/>
+      <c r="E81" s="33"/>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A82" s="36"/>
-      <c r="D82" s="32"/>
-      <c r="E82" s="32"/>
+      <c r="A82" s="37"/>
+      <c r="B82" s="4"/>
+      <c r="D82" s="33"/>
+      <c r="E82" s="33"/>
+      <c r="F82" s="28"/>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A83" s="36"/>
-      <c r="D83" s="32"/>
-      <c r="E83" s="32"/>
+      <c r="A83" s="37"/>
+      <c r="D83" s="33"/>
+      <c r="E83" s="33"/>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A84" s="36"/>
-      <c r="D84" s="32"/>
-      <c r="E84" s="32"/>
+      <c r="A84" s="37"/>
+      <c r="D84" s="33"/>
+      <c r="E84" s="33"/>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A85" s="36"/>
-      <c r="D85" s="32"/>
-      <c r="E85" s="32"/>
+      <c r="A85" s="37"/>
+      <c r="D85" s="33"/>
+      <c r="E85" s="33"/>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A86" s="36"/>
-      <c r="D86" s="32"/>
-      <c r="E86" s="32"/>
+      <c r="A86" s="37"/>
+      <c r="D86" s="33"/>
+      <c r="E86" s="33"/>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A87" s="36"/>
-      <c r="B87" s="3"/>
-      <c r="D87" s="32"/>
-      <c r="E87" s="32"/>
-      <c r="F87" s="27"/>
+      <c r="A87" s="37"/>
+      <c r="D87" s="33"/>
+      <c r="E87" s="33"/>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A88" s="36"/>
-      <c r="D88" s="32"/>
-      <c r="E88" s="32"/>
+      <c r="A88" s="37"/>
+      <c r="B88" s="4"/>
+      <c r="D88" s="33"/>
+      <c r="E88" s="33"/>
+      <c r="F88" s="28"/>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A89" s="36"/>
-      <c r="D89" s="32"/>
-      <c r="E89" s="32"/>
+      <c r="A89" s="37"/>
+      <c r="D89" s="33"/>
+      <c r="E89" s="33"/>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A90" s="36"/>
-      <c r="D90" s="32"/>
-      <c r="E90" s="32"/>
+      <c r="A90" s="37"/>
+      <c r="D90" s="33"/>
+      <c r="E90" s="33"/>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A91" s="36"/>
+      <c r="A91" s="37"/>
+      <c r="D91" s="33"/>
+      <c r="E91" s="33"/>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A92" s="36"/>
-      <c r="D92" s="32"/>
-      <c r="E92" s="32"/>
+      <c r="A92" s="37"/>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A93" s="36"/>
-      <c r="D93" s="32"/>
-      <c r="E93" s="32"/>
+      <c r="A93" s="37"/>
+      <c r="D93" s="33"/>
+      <c r="E93" s="33"/>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A94" s="36"/>
-      <c r="D94" s="32"/>
-      <c r="E94" s="32"/>
+      <c r="A94" s="37"/>
+      <c r="D94" s="33"/>
+      <c r="E94" s="33"/>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A95" s="36"/>
-      <c r="D95" s="32"/>
-      <c r="E95" s="32"/>
+      <c r="A95" s="37"/>
+      <c r="D95" s="33"/>
+      <c r="E95" s="33"/>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A96" s="36"/>
-      <c r="D96" s="32"/>
-      <c r="E96" s="32"/>
-    </row>
-    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="D97" s="32"/>
-      <c r="E97" s="32"/>
+      <c r="A96" s="37"/>
+      <c r="D96" s="33"/>
+      <c r="E96" s="33"/>
+    </row>
+    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A97" s="37"/>
+      <c r="D97" s="33"/>
+      <c r="E97" s="33"/>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="D98" s="32"/>
-      <c r="E98" s="32"/>
+      <c r="D98" s="33"/>
+      <c r="E98" s="33"/>
+    </row>
+    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="D99" s="33"/>
+      <c r="E99" s="33"/>
     </row>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="I2:R21"/>
+    <mergeCell ref="I2:R22"/>
     <mergeCell ref="E4:G6"/>
   </mergeCells>
-  <conditionalFormatting sqref="G13:G91">
+  <conditionalFormatting sqref="G13:G92">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>"COMPLETED"</formula>
     </cfRule>
@@ -2528,7 +2557,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="G13:G91" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="G13:G92" type="list">
       <formula1>"IN PROGRESS,PAUSED,COMPLETED"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>